<commit_message>
update .xlsx template sheet
</commit_message>
<xml_diff>
--- a/ignition_tag_tool_template.xlsx
+++ b/ignition_tag_tool_template.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Tools\IgnitionTagTool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E09AEBD1-99DE-45B7-8C1B-5ACC58D41AFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C5E5D3C-E072-4F60-A41A-939DC6AEA049}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="tagImport" sheetId="1" r:id="rId1"/>
-    <sheet name="udtImport" sheetId="2" r:id="rId2"/>
+    <sheet name="DEVICE_LIST" sheetId="1" r:id="rId1"/>
+    <sheet name="UDT_LIST" sheetId="2" r:id="rId2"/>
     <sheet name="simple UDTs" sheetId="3" r:id="rId3"/>
     <sheet name="Sheet5" sheetId="7" r:id="rId4"/>
     <sheet name="multi-tag UDT" sheetId="4" r:id="rId5"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="685" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="700" uniqueCount="176">
   <si>
     <t>Datatype</t>
   </si>
@@ -564,6 +564,24 @@
   </si>
   <si>
     <t>equal</t>
+  </si>
+  <si>
+    <t>TypeId</t>
+  </si>
+  <si>
+    <t>test_a_bool</t>
+  </si>
+  <si>
+    <t>this is a test a bool udt</t>
+  </si>
+  <si>
+    <t>test_imports/A_Bool</t>
+  </si>
+  <si>
+    <t>Test Device Name</t>
+  </si>
+  <si>
+    <t>:udtTagName</t>
   </si>
 </sst>
 </file>
@@ -942,18 +960,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:T3"/>
+  <dimension ref="A1:T5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.140625" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="25.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="17" style="2" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="26.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.85546875" style="2" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="8.140625" style="2" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9.5703125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="11.5703125" bestFit="1" customWidth="1"/>
@@ -1089,6 +1106,58 @@
       <c r="K3" t="s">
         <v>163</v>
       </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" t="s">
+        <v>170</v>
+      </c>
+      <c r="D4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" t="s">
+        <v>24</v>
+      </c>
+      <c r="G4" t="s">
+        <v>33</v>
+      </c>
+      <c r="H4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>171</v>
+      </c>
+      <c r="B5" t="s">
+        <v>172</v>
+      </c>
+      <c r="C5" t="s">
+        <v>173</v>
+      </c>
+      <c r="D5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E5" t="s">
+        <v>31</v>
+      </c>
+      <c r="F5" t="s">
+        <v>174</v>
+      </c>
+      <c r="G5"/>
+      <c r="H5"/>
+      <c r="I5"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
update template sheet for new parameter binding method
</commit_message>
<xml_diff>
--- a/ignition_tag_tool_template.xlsx
+++ b/ignition_tag_tool_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Tools\IgnitionTagTool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32054E0C-D9FE-4E52-8A16-4CC18F9622ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E36045F-233F-4BFA-A85D-77831A8E1B79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-12330" yWindow="-16320" windowWidth="29040" windowHeight="15720" tabRatio="729" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DEVICE_LIST" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="783" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="867" uniqueCount="170">
   <si>
     <t>Datatype</t>
   </si>
@@ -544,9 +544,6 @@
     <t>TagGroup</t>
   </si>
   <si>
-    <t>test_group</t>
-  </si>
-  <si>
     <t>this is the format for importing a UDT type instance</t>
   </si>
   <si>
@@ -559,61 +556,7 @@
     <t>test</t>
   </si>
   <si>
-    <t>test w mulitple params</t>
-  </si>
-  <si>
-    <t>P2</t>
-  </si>
-  <si>
-    <t>Param4_Name</t>
-  </si>
-  <si>
-    <t>Param4_DataType</t>
-  </si>
-  <si>
-    <t>Param4_Value</t>
-  </si>
-  <si>
-    <t>Param5_Name</t>
-  </si>
-  <si>
-    <t>Param5_DataType</t>
-  </si>
-  <si>
-    <t>Param5_Value</t>
-  </si>
-  <si>
-    <t>P4</t>
-  </si>
-  <si>
-    <t>P5</t>
-  </si>
-  <si>
     <t>test_tag</t>
-  </si>
-  <si>
-    <t>test_udt</t>
-  </si>
-  <si>
-    <t>{P1} PV Status</t>
-  </si>
-  <si>
-    <t>test_bool</t>
-  </si>
-  <si>
-    <t>test_float</t>
-  </si>
-  <si>
-    <t>test floating point</t>
-  </si>
-  <si>
-    <t>test_int</t>
-  </si>
-  <si>
-    <t>test int</t>
-  </si>
-  <si>
-    <t>PLC.test_bool</t>
   </si>
   <si>
     <t>test_c_bool</t>
@@ -1009,10 +952,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V5"/>
+  <dimension ref="A1:V6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="27.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.85546875" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12" style="2" customWidth="1"/>
     <col min="3" max="3" width="16.5703125" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="25.5703125" style="2" bestFit="1" customWidth="1"/>
@@ -1040,7 +983,7 @@
         <v>56</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>161</v>
@@ -1099,10 +1042,10 @@
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>177</v>
+        <v>166</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>4</v>
@@ -1114,59 +1057,27 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="B4" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C4" t="s">
         <v>156</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E4" t="s">
         <v>22</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F4" t="s">
         <v>23</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G4" t="s">
         <v>24</v>
-      </c>
-      <c r="H3" t="s">
-        <v>33</v>
-      </c>
-      <c r="I3" t="s">
-        <v>34</v>
-      </c>
-      <c r="J3" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>157</v>
-      </c>
-      <c r="B4" t="s">
-        <v>166</v>
-      </c>
-      <c r="C4" t="s">
-        <v>147</v>
-      </c>
-      <c r="D4" t="s">
-        <v>158</v>
-      </c>
-      <c r="E4" t="s">
-        <v>36</v>
-      </c>
-      <c r="F4" t="s">
-        <v>31</v>
-      </c>
-      <c r="G4" t="s">
-        <v>159</v>
       </c>
       <c r="H4"/>
       <c r="I4"/>
@@ -1174,36 +1085,62 @@
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>186</v>
-      </c>
-      <c r="B5" t="s">
-        <v>166</v>
+        <v>157</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>165</v>
       </c>
       <c r="C5" t="s">
-        <v>25</v>
+        <v>147</v>
       </c>
       <c r="D5" t="s">
-        <v>188</v>
-      </c>
-      <c r="E5"/>
-      <c r="F5"/>
-      <c r="G5"/>
+        <v>158</v>
+      </c>
+      <c r="E5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F5" t="s">
+        <v>31</v>
+      </c>
+      <c r="G5" t="s">
+        <v>159</v>
+      </c>
       <c r="H5"/>
       <c r="I5"/>
       <c r="J5"/>
-      <c r="K5"/>
-      <c r="L5"/>
-      <c r="P5"/>
-      <c r="Q5"/>
-      <c r="R5"/>
-      <c r="S5"/>
-      <c r="T5"/>
-      <c r="U5"/>
-      <c r="V5"/>
+    </row>
+    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>167</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="C6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" t="s">
+        <v>169</v>
+      </c>
+      <c r="E6"/>
+      <c r="F6"/>
+      <c r="G6"/>
+      <c r="H6"/>
+      <c r="I6"/>
+      <c r="J6"/>
+      <c r="K6"/>
+      <c r="L6"/>
+      <c r="P6"/>
+      <c r="Q6"/>
+      <c r="R6"/>
+      <c r="S6"/>
+      <c r="T6"/>
+      <c r="U6"/>
+      <c r="V6"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G6:G1048576 F3:F4" xr:uid="{B930CA3F-E96C-4EF7-B397-B0878359C6C5}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G7:G1048576 F4:F5" xr:uid="{B930CA3F-E96C-4EF7-B397-B0878359C6C5}">
       <formula1>"Boolean,DateTime,Float4,Float8,Int4,Int8,String"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1214,17 +1151,17 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3BC81CAD-EB70-4DE8-9674-E15A5C8680D9}">
-  <dimension ref="A1:U31"/>
+  <dimension ref="A1:T31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="21.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="36.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="26.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="17.5703125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.85546875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="20" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="14.7109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="17" style="1" bestFit="1" customWidth="1"/>
@@ -1242,11 +1179,11 @@
     <col min="24" max="24" width="13.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" t="s">
         <v>4</v>
       </c>
       <c r="C1" s="2" t="s">
@@ -1258,224 +1195,166 @@
       <c r="E1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="O1" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="P1" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="Q1" s="2" t="s">
-        <v>174</v>
-      </c>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
+      <c r="M1" s="2"/>
+      <c r="N1" s="2"/>
+      <c r="O1" s="2"/>
+      <c r="P1" s="2"/>
+      <c r="Q1" s="2"/>
       <c r="R1" s="2"/>
       <c r="S1" s="2"/>
       <c r="T1" s="2"/>
-      <c r="U1" s="2"/>
-    </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>167</v>
+    </row>
+    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B2" t="s">
+        <v>58</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>30</v>
+        <v>59</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>168</v>
-      </c>
+        <v>137</v>
+      </c>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
-      <c r="J2" s="2" t="s">
-        <v>31</v>
-      </c>
+      <c r="J2" s="2"/>
       <c r="K2" s="2"/>
-      <c r="L2" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>137</v>
-      </c>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
       <c r="N2" s="2"/>
-      <c r="O2" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="P2" s="2" t="s">
-        <v>31</v>
-      </c>
+      <c r="O2" s="2"/>
+      <c r="P2" s="2"/>
       <c r="Q2" s="2"/>
       <c r="R2" s="2"/>
       <c r="S2" s="2"/>
       <c r="T2" s="2"/>
-      <c r="U2" s="2"/>
-    </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+    </row>
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>56</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>161</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>21</v>
+        <v>4</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>39</v>
+        <v>12</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>6</v>
+        <v>153</v>
       </c>
       <c r="P3" s="2" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R3" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="S3" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="T3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="U3" s="2" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="C4" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>179</v>
+      <c r="S3" s="2"/>
+      <c r="T3" s="2"/>
+    </row>
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="G4" s="2"/>
-      <c r="H4" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="J4" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="K4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
+      <c r="K4" s="2" t="s">
+        <v>136</v>
+      </c>
       <c r="L4" s="2"/>
       <c r="M4" s="2"/>
-      <c r="N4" s="2" t="b">
-        <v>0</v>
-      </c>
+      <c r="N4" s="2"/>
       <c r="O4" s="2"/>
       <c r="P4" s="2"/>
       <c r="Q4" s="2"/>
       <c r="R4" s="2"/>
       <c r="S4" s="2"/>
       <c r="T4" s="2"/>
-      <c r="U4" s="2"/>
-    </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>181</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="C5" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>182</v>
+    </row>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G5" s="2"/>
-      <c r="H5" s="3"/>
+        <v>15</v>
+      </c>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="H5" s="2"/>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
-      <c r="K5" s="2"/>
+      <c r="K5" s="2" t="s">
+        <v>136</v>
+      </c>
       <c r="L5" s="2"/>
       <c r="M5" s="2"/>
       <c r="N5" s="2"/>
@@ -1485,32 +1364,30 @@
       <c r="R5" s="2"/>
       <c r="S5" s="2"/>
       <c r="T5" s="2"/>
-      <c r="U5" s="2"/>
-    </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="C6" s="3" t="b">
-        <v>0</v>
+    </row>
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>62</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>90</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>184</v>
+        <v>27</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G6" s="2"/>
+        <v>15</v>
+      </c>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2" t="s">
+        <v>110</v>
+      </c>
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
-      <c r="K6" s="2"/>
+      <c r="K6" s="2" t="s">
+        <v>136</v>
+      </c>
       <c r="L6" s="2"/>
       <c r="M6" s="2"/>
       <c r="N6" s="2"/>
@@ -1520,67 +1397,63 @@
       <c r="R6" s="2"/>
       <c r="S6" s="2"/>
       <c r="T6" s="2"/>
-      <c r="U6" s="2"/>
-    </row>
-    <row r="7" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C7" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>149</v>
+    </row>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>63</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I7" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="J7" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="N7" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O7" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="P7" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="Q7" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="R7" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="S7" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="T7" s="2" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="L7" s="2"/>
+      <c r="M7" s="2"/>
+      <c r="N7" s="2"/>
+      <c r="O7" s="2"/>
+      <c r="P7" s="2"/>
+      <c r="Q7" s="2"/>
+      <c r="R7" s="2"/>
+      <c r="S7" s="2"/>
+      <c r="T7" s="2"/>
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>64</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
+      <c r="G8" s="2" t="s">
+        <v>112</v>
+      </c>
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
+      <c r="K8" s="2" t="s">
+        <v>136</v>
+      </c>
       <c r="L8" s="2"/>
       <c r="M8" s="2"/>
       <c r="N8" s="2"/>
@@ -1590,20 +1463,28 @@
       <c r="R8" s="2"/>
       <c r="S8" s="2"/>
       <c r="T8" s="2"/>
-      <c r="U8" s="2"/>
-    </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
+    </row>
+    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>65</v>
+      </c>
       <c r="C9" s="2"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="2"/>
+      <c r="D9" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="3"/>
+      <c r="G9" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="H9" s="2"/>
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
-      <c r="K9" s="2"/>
+      <c r="K9" s="2" t="s">
+        <v>136</v>
+      </c>
       <c r="L9" s="2"/>
       <c r="M9" s="2"/>
       <c r="N9" s="2"/>
@@ -1613,20 +1494,28 @@
       <c r="R9" s="2"/>
       <c r="S9" s="2"/>
       <c r="T9" s="2"/>
-      <c r="U9" s="2"/>
-    </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2"/>
+    </row>
+    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>66</v>
+      </c>
       <c r="C10" s="2"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="2"/>
+      <c r="D10" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
-      <c r="H10" s="3"/>
+      <c r="G10" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="H10" s="2"/>
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
-      <c r="K10" s="2"/>
+      <c r="K10" s="2" t="s">
+        <v>136</v>
+      </c>
       <c r="L10" s="2"/>
       <c r="M10" s="2"/>
       <c r="N10" s="2"/>
@@ -1636,20 +1525,28 @@
       <c r="R10" s="2"/>
       <c r="S10" s="2"/>
       <c r="T10" s="2"/>
-      <c r="U10" s="2"/>
-    </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
+    </row>
+    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>67</v>
+      </c>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
+      <c r="G11" s="2" t="s">
+        <v>115</v>
+      </c>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
-      <c r="K11" s="2"/>
+      <c r="K11" s="2" t="s">
+        <v>136</v>
+      </c>
       <c r="L11" s="2"/>
       <c r="M11" s="2"/>
       <c r="N11" s="2"/>
@@ -1659,20 +1556,30 @@
       <c r="R11" s="2"/>
       <c r="S11" s="2"/>
       <c r="T11" s="2"/>
-      <c r="U11" s="2"/>
-    </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
+    </row>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>68</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
+      <c r="G12" s="2" t="s">
+        <v>116</v>
+      </c>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
-      <c r="K12" s="2"/>
+      <c r="K12" s="2" t="s">
+        <v>136</v>
+      </c>
       <c r="L12" s="2"/>
       <c r="M12" s="2"/>
       <c r="N12" s="2"/>
@@ -1682,20 +1589,30 @@
       <c r="R12" s="2"/>
       <c r="S12" s="2"/>
       <c r="T12" s="2"/>
-      <c r="U12" s="2"/>
-    </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="2"/>
+    </row>
+    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>69</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
+      <c r="G13" s="2" t="s">
+        <v>117</v>
+      </c>
       <c r="H13" s="2"/>
       <c r="I13" s="2"/>
       <c r="J13" s="2"/>
-      <c r="K13" s="2"/>
+      <c r="K13" s="2" t="s">
+        <v>136</v>
+      </c>
       <c r="L13" s="2"/>
       <c r="M13" s="2"/>
       <c r="N13" s="2"/>
@@ -1705,20 +1622,30 @@
       <c r="R13" s="2"/>
       <c r="S13" s="2"/>
       <c r="T13" s="2"/>
-      <c r="U13" s="2"/>
-    </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="2"/>
+    </row>
+    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>70</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
-      <c r="H14" s="3"/>
+      <c r="G14" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="H14" s="2"/>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
-      <c r="K14" s="2"/>
+      <c r="K14" s="2" t="s">
+        <v>136</v>
+      </c>
       <c r="L14" s="2"/>
       <c r="M14" s="2"/>
       <c r="N14" s="2"/>
@@ -1728,20 +1655,30 @@
       <c r="R14" s="2"/>
       <c r="S14" s="2"/>
       <c r="T14" s="2"/>
-      <c r="U14" s="2"/>
-    </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="2"/>
+    </row>
+    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>71</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="3"/>
+      <c r="G15" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="H15" s="2"/>
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
-      <c r="K15" s="2"/>
+      <c r="K15" s="2" t="s">
+        <v>136</v>
+      </c>
       <c r="L15" s="2"/>
       <c r="M15" s="2"/>
       <c r="N15" s="2"/>
@@ -1751,20 +1688,30 @@
       <c r="R15" s="2"/>
       <c r="S15" s="2"/>
       <c r="T15" s="2"/>
-      <c r="U15" s="2"/>
-    </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="3"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
+    </row>
+    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>72</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="F16" s="2"/>
-      <c r="G16" s="2"/>
+      <c r="G16" s="2" t="s">
+        <v>120</v>
+      </c>
       <c r="H16" s="2"/>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
-      <c r="K16" s="2"/>
+      <c r="K16" s="2" t="s">
+        <v>136</v>
+      </c>
       <c r="L16" s="2"/>
       <c r="M16" s="2"/>
       <c r="N16" s="2"/>
@@ -1774,20 +1721,28 @@
       <c r="R16" s="2"/>
       <c r="S16" s="2"/>
       <c r="T16" s="2"/>
-      <c r="U16" s="2"/>
-    </row>
-    <row r="17" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A17" s="2"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
+    </row>
+    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>73</v>
+      </c>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="F17" s="2"/>
-      <c r="G17" s="2"/>
+      <c r="G17" s="2" t="s">
+        <v>121</v>
+      </c>
       <c r="H17" s="2"/>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
-      <c r="K17" s="2"/>
+      <c r="K17" s="2" t="s">
+        <v>136</v>
+      </c>
       <c r="L17" s="2"/>
       <c r="M17" s="2"/>
       <c r="N17" s="2"/>
@@ -1797,20 +1752,28 @@
       <c r="R17" s="2"/>
       <c r="S17" s="2"/>
       <c r="T17" s="2"/>
-      <c r="U17" s="2"/>
-    </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A18" s="2"/>
-      <c r="B18" s="2"/>
+    </row>
+    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>74</v>
+      </c>
       <c r="C18" s="2"/>
-      <c r="D18" s="3"/>
-      <c r="E18" s="2"/>
+      <c r="D18" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
+      <c r="G18" s="2" t="s">
+        <v>122</v>
+      </c>
       <c r="H18" s="2"/>
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
-      <c r="K18" s="2"/>
+      <c r="K18" s="2" t="s">
+        <v>136</v>
+      </c>
       <c r="L18" s="2"/>
       <c r="M18" s="2"/>
       <c r="N18" s="2"/>
@@ -1820,20 +1783,28 @@
       <c r="R18" s="2"/>
       <c r="S18" s="2"/>
       <c r="T18" s="2"/>
-      <c r="U18" s="2"/>
-    </row>
-    <row r="19" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A19" s="2"/>
-      <c r="B19" s="2"/>
+    </row>
+    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>75</v>
+      </c>
       <c r="C19" s="2"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="2"/>
+      <c r="D19" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="F19" s="2"/>
-      <c r="G19" s="2"/>
-      <c r="H19" s="3"/>
+      <c r="G19" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="H19" s="2"/>
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
-      <c r="K19" s="2"/>
+      <c r="K19" s="2" t="s">
+        <v>136</v>
+      </c>
       <c r="L19" s="2"/>
       <c r="M19" s="2"/>
       <c r="N19" s="2"/>
@@ -1843,20 +1814,30 @@
       <c r="R19" s="2"/>
       <c r="S19" s="2"/>
       <c r="T19" s="2"/>
-      <c r="U19" s="2"/>
-    </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A20" s="2"/>
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="3"/>
-      <c r="E20" s="2"/>
+    </row>
+    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>76</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>16</v>
+      </c>
       <c r="F20" s="2"/>
-      <c r="G20" s="2"/>
-      <c r="H20" s="3"/>
+      <c r="G20" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="H20" s="2"/>
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
-      <c r="K20" s="2"/>
+      <c r="K20" s="2" t="s">
+        <v>136</v>
+      </c>
       <c r="L20" s="2"/>
       <c r="M20" s="2"/>
       <c r="N20" s="2"/>
@@ -1866,20 +1847,30 @@
       <c r="R20" s="2"/>
       <c r="S20" s="2"/>
       <c r="T20" s="2"/>
-      <c r="U20" s="2"/>
-    </row>
-    <row r="21" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A21" s="2"/>
-      <c r="B21" s="2"/>
-      <c r="C21" s="3"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
+    </row>
+    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>77</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>16</v>
+      </c>
       <c r="F21" s="2"/>
-      <c r="G21" s="2"/>
+      <c r="G21" s="2" t="s">
+        <v>125</v>
+      </c>
       <c r="H21" s="2"/>
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
-      <c r="K21" s="2"/>
+      <c r="K21" s="2" t="s">
+        <v>136</v>
+      </c>
       <c r="L21" s="2"/>
       <c r="M21" s="2"/>
       <c r="N21" s="2"/>
@@ -1889,20 +1880,28 @@
       <c r="R21" s="2"/>
       <c r="S21" s="2"/>
       <c r="T21" s="2"/>
-      <c r="U21" s="2"/>
-    </row>
-    <row r="22" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A22" s="2"/>
-      <c r="B22" s="2"/>
-      <c r="C22" s="3"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
+    </row>
+    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>78</v>
+      </c>
+      <c r="C22" s="2"/>
+      <c r="D22" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>16</v>
+      </c>
       <c r="F22" s="2"/>
-      <c r="G22" s="2"/>
+      <c r="G22" s="2" t="s">
+        <v>126</v>
+      </c>
       <c r="H22" s="2"/>
       <c r="I22" s="2"/>
       <c r="J22" s="2"/>
-      <c r="K22" s="2"/>
+      <c r="K22" s="2" t="s">
+        <v>136</v>
+      </c>
       <c r="L22" s="2"/>
       <c r="M22" s="2"/>
       <c r="N22" s="2"/>
@@ -1912,20 +1911,30 @@
       <c r="R22" s="2"/>
       <c r="S22" s="2"/>
       <c r="T22" s="2"/>
-      <c r="U22" s="2"/>
-    </row>
-    <row r="23" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A23" s="2"/>
-      <c r="B23" s="2"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="3"/>
-      <c r="E23" s="2"/>
+    </row>
+    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>79</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>16</v>
+      </c>
       <c r="F23" s="2"/>
-      <c r="G23" s="2"/>
+      <c r="G23" s="2" t="s">
+        <v>127</v>
+      </c>
       <c r="H23" s="2"/>
       <c r="I23" s="2"/>
       <c r="J23" s="2"/>
-      <c r="K23" s="2"/>
+      <c r="K23" s="2" t="s">
+        <v>136</v>
+      </c>
       <c r="L23" s="2"/>
       <c r="M23" s="2"/>
       <c r="N23" s="2"/>
@@ -1935,20 +1944,28 @@
       <c r="R23" s="2"/>
       <c r="S23" s="2"/>
       <c r="T23" s="2"/>
-      <c r="U23" s="2"/>
-    </row>
-    <row r="24" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A24" s="2"/>
-      <c r="B24" s="2"/>
+    </row>
+    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>80</v>
+      </c>
       <c r="C24" s="2"/>
-      <c r="D24" s="3"/>
-      <c r="E24" s="2"/>
+      <c r="D24" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>16</v>
+      </c>
       <c r="F24" s="2"/>
-      <c r="G24" s="2"/>
-      <c r="H24" s="3"/>
+      <c r="G24" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="H24" s="2"/>
       <c r="I24" s="2"/>
       <c r="J24" s="2"/>
-      <c r="K24" s="2"/>
+      <c r="K24" s="2" t="s">
+        <v>136</v>
+      </c>
       <c r="L24" s="2"/>
       <c r="M24" s="2"/>
       <c r="N24" s="2"/>
@@ -1958,20 +1975,30 @@
       <c r="R24" s="2"/>
       <c r="S24" s="2"/>
       <c r="T24" s="2"/>
-      <c r="U24" s="2"/>
-    </row>
-    <row r="25" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A25" s="2"/>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="4"/>
+    </row>
+    <row r="25" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>81</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>13</v>
+      </c>
       <c r="F25" s="2"/>
-      <c r="G25" s="2"/>
+      <c r="G25" s="2" t="s">
+        <v>129</v>
+      </c>
       <c r="H25" s="2"/>
       <c r="I25" s="2"/>
       <c r="J25" s="2"/>
-      <c r="K25" s="2"/>
+      <c r="K25" s="2" t="s">
+        <v>136</v>
+      </c>
       <c r="L25" s="2"/>
       <c r="M25" s="2"/>
       <c r="N25" s="2"/>
@@ -1981,30 +2008,212 @@
       <c r="R25" s="2"/>
       <c r="S25" s="2"/>
       <c r="T25" s="2"/>
-      <c r="U25" s="2"/>
-    </row>
-    <row r="26" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="27" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="29" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="D29" s="3"/>
-      <c r="H29" s="3"/>
-    </row>
-    <row r="30" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="H30" s="1"/>
-      <c r="K30"/>
-    </row>
-    <row r="31" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="H31" s="1"/>
-      <c r="K31"/>
+    </row>
+    <row r="26" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>82</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F26" s="2"/>
+      <c r="G26" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="H26" s="2"/>
+      <c r="I26" s="2"/>
+      <c r="J26" s="2"/>
+      <c r="K26" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="L26" s="2"/>
+      <c r="M26" s="2"/>
+      <c r="N26" s="2"/>
+      <c r="O26" s="2"/>
+      <c r="P26" s="2"/>
+      <c r="Q26" s="2"/>
+      <c r="R26" s="2"/>
+      <c r="S26" s="2"/>
+      <c r="T26" s="2"/>
+    </row>
+    <row r="27" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>83</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F27" s="2"/>
+      <c r="G27" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="H27" s="2"/>
+      <c r="I27" s="2"/>
+      <c r="J27" s="2"/>
+      <c r="K27" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="L27" s="2"/>
+      <c r="M27" s="2"/>
+      <c r="N27" s="2"/>
+      <c r="O27" s="2"/>
+      <c r="P27" s="2"/>
+      <c r="Q27" s="2"/>
+      <c r="R27" s="2"/>
+      <c r="S27" s="2"/>
+      <c r="T27" s="2"/>
+    </row>
+    <row r="28" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>84</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F28" s="2"/>
+      <c r="G28" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="H28" s="2"/>
+      <c r="I28" s="2"/>
+      <c r="J28" s="2"/>
+      <c r="K28" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="L28" s="2"/>
+      <c r="M28" s="2"/>
+      <c r="N28" s="2"/>
+      <c r="O28" s="2"/>
+      <c r="P28" s="2"/>
+      <c r="Q28" s="2"/>
+      <c r="R28" s="2"/>
+      <c r="S28" s="2"/>
+      <c r="T28" s="2"/>
+    </row>
+    <row r="29" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>85</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F29" s="2"/>
+      <c r="G29" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="H29" s="2"/>
+      <c r="I29" s="2"/>
+      <c r="J29" s="2"/>
+      <c r="K29" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="L29" s="2"/>
+      <c r="M29" s="2"/>
+      <c r="N29" s="2"/>
+      <c r="O29" s="2"/>
+      <c r="P29" s="2"/>
+      <c r="Q29" s="2"/>
+      <c r="R29" s="2"/>
+      <c r="S29" s="2"/>
+      <c r="T29" s="2"/>
+    </row>
+    <row r="30" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>86</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F30" s="2"/>
+      <c r="G30" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="H30" s="2"/>
+      <c r="I30" s="2"/>
+      <c r="J30" s="2"/>
+      <c r="K30" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="L30" s="2"/>
+      <c r="M30" s="2"/>
+      <c r="N30" s="2"/>
+      <c r="O30" s="2"/>
+      <c r="P30" s="2"/>
+      <c r="Q30" s="2"/>
+      <c r="R30" s="2"/>
+      <c r="S30" s="2"/>
+      <c r="T30" s="2"/>
+    </row>
+    <row r="31" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>87</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F31" s="2"/>
+      <c r="G31" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="H31" s="2"/>
+      <c r="I31" s="2"/>
+      <c r="J31" s="2"/>
+      <c r="K31" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="L31" s="2"/>
+      <c r="M31" s="2"/>
+      <c r="N31" s="2"/>
+      <c r="O31" s="2"/>
+      <c r="P31" s="2"/>
+      <c r="Q31" s="2"/>
+      <c r="R31" s="2"/>
+      <c r="S31" s="2"/>
+      <c r="T31" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E29:E31 E4:E5 E9:E10 E14:E15 E19:E20 E24 E7" xr:uid="{725D62A1-D8DF-4987-A02B-85F6B1F95203}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4:D31" xr:uid="{4E0B38AD-AD7A-45DC-B44D-F4769DC8AC52}">
       <formula1>"memory,opc"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4:F5 F9:F10 F14:F15 F19:F20 F24 F29 F7" xr:uid="{0EA0B629-E0CC-483E-9F19-101D52AAA309}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4:E5" xr:uid="{7D6CCEE6-4206-4732-A679-1B74F1BBC2BE}">
       <formula1>"Boolean,Int1,Int2,Int4,Int8,Float4,Float8,String"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2023,7 +2232,7 @@
         <v>56</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>161</v>
@@ -2087,7 +2296,7 @@
         <v>160</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C2" t="s">
         <v>156</v>
@@ -2154,7 +2363,7 @@
         <v>160</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C1" t="s">
         <v>156</v>
@@ -2195,7 +2404,7 @@
         <v>157</v>
       </c>
       <c r="B2" t="s">
-        <v>187</v>
+        <v>168</v>
       </c>
       <c r="C2" t="s">
         <v>147</v>
@@ -2224,18 +2433,18 @@
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>186</v>
+        <v>167</v>
       </c>
       <c r="C3" t="s">
         <v>37</v>
       </c>
       <c r="D3" t="s">
-        <v>188</v>
+        <v>169</v>
       </c>
     </row>
     <row r="11" spans="1:22" x14ac:dyDescent="0.25">
       <c r="C11" s="6" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
   </sheetData>
@@ -2255,22 +2464,22 @@
   <cols>
     <col min="1" max="1" width="10.42578125" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="7.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11" style="2" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="16.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="17.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12" style="2" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="14" style="2" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="11.5703125" style="2" bestFit="1" customWidth="1"/>
     <col min="20" max="21" width="14" style="2" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="14" bestFit="1" customWidth="1"/>
@@ -2335,96 +2544,81 @@
         <v>161</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>21</v>
+        <v>4</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>39</v>
+        <v>12</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>6</v>
+        <v>153</v>
       </c>
       <c r="P3" s="2" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R3" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="S3" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="T3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="U3" s="2" t="s">
         <v>9</v>
       </c>
+      <c r="S3"/>
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C4" s="2" t="b">
+      <c r="C4" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K4" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="D4" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="H4" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="J4" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="N4" s="2" t="b">
-        <v>1</v>
-      </c>
+      <c r="S4"/>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="D5" s="3"/>
       <c r="E5" s="2"/>
       <c r="H5" s="3"/>
+      <c r="U5"/>
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
@@ -2451,6 +2645,7 @@
       <c r="H6" s="2" t="s">
         <v>35</v>
       </c>
+      <c r="U6"/>
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
@@ -2474,6 +2669,7 @@
       <c r="G7" s="2" t="s">
         <v>31</v>
       </c>
+      <c r="U7"/>
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
@@ -2482,92 +2678,76 @@
       <c r="B8" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D8" s="3" t="s">
+      <c r="C8" s="3" t="s">
         <v>4</v>
       </c>
+      <c r="D8" s="2" t="s">
+        <v>2</v>
+      </c>
       <c r="E8" s="2" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>39</v>
+        <v>12</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="O8" s="2" t="s">
-        <v>6</v>
+        <v>153</v>
       </c>
       <c r="P8" s="2" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="Q8" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R8" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="S8" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="T8" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="U8" s="2" t="s">
         <v>9</v>
       </c>
+      <c r="T8"/>
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="D9" s="3" t="s">
+      <c r="C9" s="3" t="s">
         <v>140</v>
       </c>
+      <c r="D9" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="E9" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F9" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="H9" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I9" s="2" t="s">
+      <c r="G9" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="J9" s="2" t="b">
+      <c r="K9" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="N9" s="2" t="b">
-        <v>0</v>
-      </c>
+      <c r="T9"/>
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="D10" s="3"/>
@@ -2645,61 +2825,52 @@
       <c r="B13" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="C13" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D13" s="3" t="s">
+      <c r="C13" s="3" t="s">
         <v>4</v>
       </c>
+      <c r="D13" s="2" t="s">
+        <v>2</v>
+      </c>
       <c r="E13" s="2" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>39</v>
+        <v>12</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="L13" s="2" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="O13" s="2" t="s">
-        <v>6</v>
+        <v>153</v>
       </c>
       <c r="P13" s="2" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="Q13" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R13" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="S13" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="T13" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="U13" s="2" t="s">
         <v>9</v>
       </c>
     </row>
@@ -2707,34 +2878,25 @@
       <c r="A14" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C14" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="D14" s="3" t="s">
+      <c r="C14" s="3" t="s">
         <v>140</v>
       </c>
+      <c r="D14" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="E14" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F14" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H14" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I14" s="2" t="s">
+      <c r="G14" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="J14" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="K14" s="2" t="s">
+      <c r="H14" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="L14" s="2">
+      <c r="I14" s="2">
         <v>32767</v>
       </c>
-      <c r="N14" s="2" t="b">
+      <c r="K14" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2814,61 +2976,52 @@
       <c r="B18" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="C18" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D18" s="3" t="s">
+      <c r="C18" s="3" t="s">
         <v>4</v>
       </c>
+      <c r="D18" s="2" t="s">
+        <v>2</v>
+      </c>
       <c r="E18" s="2" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>39</v>
+        <v>12</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="N18" s="2" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="O18" s="2" t="s">
-        <v>6</v>
+        <v>153</v>
       </c>
       <c r="P18" s="2" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="Q18" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R18" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="S18" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="T18" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="U18" s="2" t="s">
         <v>9</v>
       </c>
     </row>
@@ -2876,34 +3029,25 @@
       <c r="A19" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C19" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="D19" s="3" t="s">
+      <c r="C19" s="3" t="s">
         <v>140</v>
       </c>
+      <c r="D19" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="E19" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F19" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="H19" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I19" s="2" t="s">
+      <c r="G19" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="J19" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="K19" s="2" t="s">
+      <c r="H19" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="L19" s="2">
+      <c r="I19" s="2">
         <v>32767</v>
       </c>
-      <c r="N19" s="2" t="b">
+      <c r="K19" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2983,98 +3127,82 @@
       <c r="B23" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="C23" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D23" s="3" t="s">
+      <c r="C23" s="3" t="s">
         <v>4</v>
       </c>
+      <c r="D23" s="2" t="s">
+        <v>2</v>
+      </c>
       <c r="E23" s="2" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="J23" s="2" t="s">
-        <v>39</v>
+        <v>12</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="L23" s="2" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="M23" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="N23" s="2" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="O23" s="2" t="s">
-        <v>6</v>
+        <v>153</v>
       </c>
       <c r="P23" s="2" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="Q23" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R23" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="S23" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="T23" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="U23" s="2" t="s">
         <v>9</v>
       </c>
+      <c r="S23"/>
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C24" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="D24" s="3" t="s">
+      <c r="C24" s="3" t="s">
         <v>140</v>
       </c>
+      <c r="D24" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="E24" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F24" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H24" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I24" s="2" t="s">
+      <c r="G24" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="J24" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="K24" s="2" t="s">
+      <c r="H24" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="L24" s="2">
+      <c r="I24" s="2">
         <v>32767</v>
       </c>
-      <c r="N24" s="2" t="b">
+      <c r="K24" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="S24"/>
     </row>
     <row r="26" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
@@ -3133,60 +3261,51 @@
         <v>161</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>21</v>
+        <v>4</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="J28" s="2" t="s">
-        <v>39</v>
+        <v>12</v>
       </c>
       <c r="K28" s="2" t="s">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="L28" s="2" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="M28" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="N28" s="2" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="O28" s="2" t="s">
-        <v>6</v>
+        <v>153</v>
       </c>
       <c r="P28" s="2" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="Q28" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R28" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="S28" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="T28" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="U28" s="2" t="s">
         <v>9</v>
       </c>
     </row>
@@ -3194,47 +3313,38 @@
       <c r="A29" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C29" s="2" t="b">
+      <c r="C29" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K29" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="D29" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="E29" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F29" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="H29" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I29" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="J29" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="N29" s="2" t="b">
-        <v>1</v>
+      <c r="L29" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="M29" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="N29" s="2" t="s">
+        <v>151</v>
       </c>
       <c r="O29" s="2" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="P29" s="2" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="Q29" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="R29" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="S29" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="T29" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
@@ -3244,10 +3354,10 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4:F5 F9:F10 F14:F15 F19:F20 F24 F29" xr:uid="{71BB14FA-1E7A-4178-9960-9FE32EC7996F}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E24 E29 E4 F5 E9 F10 E14 F15 E19 F20" xr:uid="{71BB14FA-1E7A-4178-9960-9FE32EC7996F}">
       <formula1>"Boolean,Int1,Int2,Int4,Int8,Float4,Float8,String"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4:E5 E9:E10 E14:E15 E19:E20 E24 E29" xr:uid="{77B09903-3FB9-48BF-93D7-EE046F3B3FC0}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D24 D29 D4 E5 D9 E10 D14 E15 D19 E20" xr:uid="{77B09903-3FB9-48BF-93D7-EE046F3B3FC0}">
       <formula1>"memory,opc"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3258,32 +3368,32 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{869BECBF-17B1-47F3-867F-A545F9812257}">
-  <dimension ref="A1:U7"/>
+  <dimension ref="A1:T7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="25.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="24" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17" style="2" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17.5703125" style="2" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="30.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="30.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14" style="2" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="17" style="2" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="13.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="7.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11" style="2" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="11.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11" style="2" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="16.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="14" style="2" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="11.42578125" style="2" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="14" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>55</v>
       </c>
@@ -3318,7 +3428,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>48</v>
       </c>
@@ -3341,7 +3451,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>56</v>
       </c>
@@ -3349,138 +3459,109 @@
         <v>161</v>
       </c>
       <c r="C3" t="s">
-        <v>21</v>
-      </c>
-      <c r="D3" t="s">
         <v>4</v>
       </c>
+      <c r="D3" s="2" t="s">
+        <v>2</v>
+      </c>
       <c r="E3" s="2" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>39</v>
+        <v>12</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>6</v>
+        <v>153</v>
       </c>
       <c r="P3" s="2" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R3" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="S3" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="T3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="U3" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>49</v>
       </c>
-      <c r="C4" t="b">
+      <c r="C4" t="s">
+        <v>50</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="K4" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="D4" t="s">
-        <v>50</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="H4" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="J4" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="N4" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="U4" s="2"/>
-    </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>52</v>
       </c>
-      <c r="C5" t="b">
+      <c r="C5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="I5" s="2">
+        <v>9999</v>
+      </c>
+      <c r="K5" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="D5" t="s">
-        <v>53</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="H5" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="J5" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="L5" s="2">
-        <v>9999</v>
-      </c>
-      <c r="N5" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="U5" s="2"/>
-    </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="H6" s="3"/>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="H7" s="3"/>
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4:F7" xr:uid="{8BA1F78F-26F1-4B90-A6BA-66E569BC97E4}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F6:F7 E4:E5" xr:uid="{8BA1F78F-26F1-4B90-A6BA-66E569BC97E4}">
       <formula1>"Boolean,Int1,Int2,Int4,Int8,Float4,Float8,String"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4:E7" xr:uid="{6AFBC94E-AA4F-4B76-96FC-94BA7305CD02}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E6:E7 D4:D5" xr:uid="{6AFBC94E-AA4F-4B76-96FC-94BA7305CD02}">
       <formula1>"memory,opc"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3496,27 +3577,25 @@
   <cols>
     <col min="1" max="1" width="21.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="22.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="36.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="36.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17" style="2" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="41.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="7.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="11" style="2" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="16.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="11.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="14" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="41.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="7.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11" style="2" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="16.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="18" max="20" width="14" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>55</v>
       </c>
@@ -3533,7 +3612,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>57</v>
       </c>
@@ -3547,886 +3626,597 @@
         <v>137</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>56</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="C3" t="s">
-        <v>21</v>
+      <c r="C3" s="2" t="s">
+        <v>4</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>39</v>
+        <v>12</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>6</v>
+        <v>153</v>
       </c>
       <c r="P3" s="2" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R3" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="S3" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="T3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="U3" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>60</v>
       </c>
-      <c r="C4" t="b">
-        <v>0</v>
+      <c r="C4" s="2" t="s">
+        <v>88</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>88</v>
+        <v>27</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="H4" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I4" s="2" t="s">
+      <c r="G4" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="J4" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="N4" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="U4" s="2"/>
-    </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="K4" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>61</v>
       </c>
-      <c r="C5" t="b">
-        <v>0</v>
+      <c r="C5" s="2" t="s">
+        <v>89</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>89</v>
+        <v>27</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="H5" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I5" s="2" t="s">
+      <c r="G5" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="J5" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="N5" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="U5" s="2"/>
-    </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="K5" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>62</v>
       </c>
-      <c r="C6" t="b">
-        <v>0</v>
+      <c r="C6" s="2" t="s">
+        <v>90</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>90</v>
+        <v>27</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="H6" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I6" s="2" t="s">
+      <c r="G6" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="J6" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="N6" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="U6" s="2"/>
-    </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="K6" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>63</v>
       </c>
-      <c r="C7" t="b">
-        <v>0</v>
+      <c r="C7" s="2" t="s">
+        <v>91</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>91</v>
+        <v>27</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I7" s="2" t="s">
+      <c r="G7" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="J7" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="N7" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="U7" s="2"/>
-    </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="K7" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>64</v>
       </c>
-      <c r="C8" t="b">
-        <v>0</v>
+      <c r="C8" s="2" t="s">
+        <v>92</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>92</v>
+        <v>27</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F8" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="H8" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I8" s="2" t="s">
+      <c r="G8" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="J8" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="N8" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="U8" s="2"/>
-    </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="K8" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>65</v>
       </c>
-      <c r="C9" t="b">
-        <v>0</v>
+      <c r="D9" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F9" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="H9" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I9" s="2" t="s">
+      <c r="G9" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="J9" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="N9" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="U9" s="2"/>
-    </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="K9" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>66</v>
       </c>
-      <c r="C10" t="b">
-        <v>0</v>
+      <c r="D10" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F10" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="H10" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I10" s="2" t="s">
+      <c r="G10" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="J10" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="N10" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="U10" s="2"/>
-    </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="K10" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>67</v>
       </c>
-      <c r="C11" t="b">
-        <v>0</v>
+      <c r="D11" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F11" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="H11" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I11" s="2" t="s">
+      <c r="G11" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="J11" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="N11" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="U11" s="2"/>
-    </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="K11" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>68</v>
       </c>
-      <c r="C12" t="b">
-        <v>0</v>
+      <c r="C12" s="2" t="s">
+        <v>93</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>93</v>
+        <v>27</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F12" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="H12" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I12" s="2" t="s">
+      <c r="G12" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="J12" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="N12" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="U12" s="2"/>
-    </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="K12" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>69</v>
       </c>
-      <c r="C13" t="b">
-        <v>0</v>
+      <c r="C13" s="2" t="s">
+        <v>94</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>94</v>
+        <v>27</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F13" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="H13" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I13" s="2" t="s">
+      <c r="G13" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="J13" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="N13" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="U13" s="2"/>
-    </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="K13" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>70</v>
       </c>
-      <c r="C14" t="b">
-        <v>0</v>
+      <c r="C14" s="2" t="s">
+        <v>95</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>95</v>
+        <v>27</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F14" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="H14" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I14" s="2" t="s">
+      <c r="G14" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="J14" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="N14" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="U14" s="2"/>
-    </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="K14" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>71</v>
       </c>
-      <c r="C15" t="b">
-        <v>0</v>
+      <c r="C15" s="2" t="s">
+        <v>96</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>96</v>
+        <v>27</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F15" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="H15" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I15" s="2" t="s">
+      <c r="G15" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="J15" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="N15" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="U15" s="2"/>
-    </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="K15" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>72</v>
       </c>
-      <c r="C16" t="b">
-        <v>0</v>
+      <c r="C16" s="2" t="s">
+        <v>97</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>97</v>
+        <v>27</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F16" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="H16" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I16" s="2" t="s">
+      <c r="G16" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="J16" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="N16" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="U16" s="2"/>
+      <c r="K16" s="2" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>73</v>
       </c>
-      <c r="C17" t="b">
-        <v>0</v>
+      <c r="D17" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F17" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="H17" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I17" s="2" t="s">
+      <c r="G17" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="J17" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="N17" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="U17" s="2"/>
+      <c r="K17" s="2" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>74</v>
       </c>
-      <c r="C18" t="b">
-        <v>0</v>
+      <c r="D18" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F18" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="H18" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I18" s="2" t="s">
+      <c r="G18" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="J18" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="N18" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="U18" s="2"/>
+      <c r="K18" s="2" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>75</v>
       </c>
-      <c r="C19" t="b">
-        <v>0</v>
+      <c r="D19" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F19" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="H19" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I19" s="2" t="s">
+      <c r="G19" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="J19" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="N19" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="U19" s="2"/>
+      <c r="K19" s="2" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>76</v>
       </c>
-      <c r="C20" t="b">
-        <v>0</v>
+      <c r="C20" s="2" t="s">
+        <v>98</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>98</v>
+        <v>27</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F20" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="H20" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I20" s="2" t="s">
+      <c r="G20" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="J20" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="N20" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="U20" s="2"/>
+      <c r="K20" s="2" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>77</v>
       </c>
-      <c r="C21" t="b">
-        <v>0</v>
+      <c r="C21" s="2" t="s">
+        <v>99</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>99</v>
+        <v>27</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F21" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="H21" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I21" s="2" t="s">
+      <c r="G21" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="J21" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="N21" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="U21" s="2"/>
+      <c r="K21" s="2" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>78</v>
       </c>
-      <c r="C22" t="b">
-        <v>0</v>
+      <c r="D22" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F22" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="H22" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I22" s="2" t="s">
+      <c r="G22" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="J22" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="N22" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="U22" s="2"/>
+      <c r="K22" s="2" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>79</v>
       </c>
-      <c r="C23" t="b">
-        <v>0</v>
+      <c r="C23" s="2" t="s">
+        <v>100</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>100</v>
+        <v>27</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F23" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="H23" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I23" s="2" t="s">
+      <c r="G23" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="J23" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="N23" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="U23" s="2"/>
+      <c r="K23" s="2" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>80</v>
       </c>
-      <c r="C24" t="b">
-        <v>0</v>
+      <c r="D24" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F24" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="H24" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I24" s="2" t="s">
+      <c r="G24" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="J24" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="N24" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="U24" s="2"/>
+      <c r="K24" s="2" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>81</v>
       </c>
-      <c r="C25" t="b">
-        <v>0</v>
+      <c r="C25" s="2" t="s">
+        <v>101</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>101</v>
+        <v>27</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F25" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H25" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I25" s="2" t="s">
+      <c r="G25" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="J25" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="N25" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="U25" s="2"/>
+      <c r="K25" s="2" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>82</v>
       </c>
-      <c r="C26" t="b">
-        <v>0</v>
+      <c r="C26" s="2" t="s">
+        <v>102</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>102</v>
+        <v>27</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F26" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H26" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I26" s="2" t="s">
+      <c r="G26" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="J26" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="N26" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="U26" s="2"/>
+      <c r="K26" s="2" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>83</v>
       </c>
-      <c r="C27" t="b">
-        <v>0</v>
+      <c r="C27" s="2" t="s">
+        <v>103</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>103</v>
+        <v>27</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F27" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H27" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I27" s="2" t="s">
+      <c r="G27" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="J27" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="N27" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="U27" s="2"/>
+      <c r="K27" s="2" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>84</v>
       </c>
-      <c r="C28" t="b">
-        <v>0</v>
+      <c r="C28" s="2" t="s">
+        <v>104</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>104</v>
+        <v>27</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F28" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H28" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I28" s="2" t="s">
+      <c r="G28" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="J28" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="N28" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="U28" s="2"/>
+      <c r="K28" s="2" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>85</v>
       </c>
-      <c r="C29" t="b">
-        <v>0</v>
+      <c r="C29" s="2" t="s">
+        <v>105</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>105</v>
+        <v>27</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F29" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H29" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I29" s="2" t="s">
+      <c r="G29" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="J29" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="N29" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="U29" s="2"/>
+      <c r="K29" s="2" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>86</v>
       </c>
-      <c r="C30" t="b">
-        <v>0</v>
+      <c r="C30" s="2" t="s">
+        <v>106</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>106</v>
+        <v>27</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F30" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H30" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I30" s="2" t="s">
+      <c r="G30" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="J30" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="N30" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="U30" s="2"/>
+      <c r="K30" s="2" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>87</v>
       </c>
-      <c r="C31" t="b">
-        <v>0</v>
+      <c r="C31" s="2" t="s">
+        <v>107</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>107</v>
+        <v>27</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F31" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="H31" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I31" s="2" t="s">
+      <c r="G31" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="J31" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="N31" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="U31" s="2"/>
+      <c r="K31" s="2" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.25">
       <c r="C32"/>
@@ -4434,10 +4224,10 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4:E31" xr:uid="{E807AF82-1EFC-4484-ACFE-E263504FDBC8}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4:D31" xr:uid="{E807AF82-1EFC-4484-ACFE-E263504FDBC8}">
       <formula1>"memory,opc"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4:F5" xr:uid="{7E70ACDF-680E-474C-9B11-CD1D2D08BA1A}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4:E5" xr:uid="{7E70ACDF-680E-474C-9B11-CD1D2D08BA1A}">
       <formula1>"Boolean,Int1,Int2,Int4,Int8,Float4,Float8,String"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>